<commit_message>
Add product listing images and promo videos (AR/EN)
Images and videos are built from real screenshots of the workbook.
Also fixes dashboard chart sizing, empty-row data bars and tracker
row heights found while capturing them, and adds demo tracker rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CZ61MmEF1R8eWBdqxEbAgG
</commit_message>
<xml_diff>
--- a/budget-2027/dist/Planner-2027-AR.xlsx
+++ b/budget-2027/dist/Planner-2027-AR.xlsx
@@ -108,7 +108,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="135">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="303" uniqueCount="137">
   <si>
     <t xml:space="preserve">مخطط الميزانية والأهداف ورمضان 2027</t>
   </si>
@@ -467,6 +467,9 @@
     <t xml:space="preserve">صدقة</t>
   </si>
   <si>
+    <t xml:space="preserve">✓</t>
+  </si>
+  <si>
     <t xml:space="preserve">أيام متبقية على رمضان</t>
   </si>
   <si>
@@ -477,6 +480,9 @@
   </si>
   <si>
     <t xml:space="preserve">الفعلي في رمضان</t>
+  </si>
+  <si>
+    <t xml:space="preserve">✗</t>
   </si>
   <si>
     <t xml:space="preserve">كل المصروفات خلال رمضان</t>
@@ -1406,11 +1412,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="81907942"/>
-        <c:axId val="60049300"/>
+        <c:axId val="48488034"/>
+        <c:axId val="25957626"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="81907942"/>
+        <c:axId val="48488034"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1442,7 +1448,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="60049300"/>
+        <c:crossAx val="25957626"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1450,7 +1456,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="60049300"/>
+        <c:axId val="25957626"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1492,7 +1498,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81907942"/>
+        <c:crossAx val="48488034"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1808,11 +1814,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="29216775"/>
-        <c:axId val="62259650"/>
+        <c:axId val="3261588"/>
+        <c:axId val="29794122"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="29216775"/>
+        <c:axId val="3261588"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -1844,7 +1850,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62259650"/>
+        <c:crossAx val="29794122"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1852,7 +1858,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="62259650"/>
+        <c:axId val="29794122"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1894,7 +1900,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="29216775"/>
+        <c:crossAx val="3261588"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2287,11 +2293,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="69572257"/>
-        <c:axId val="10721836"/>
+        <c:axId val="95415480"/>
+        <c:axId val="8730332"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="69572257"/>
+        <c:axId val="95415480"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2323,7 +2329,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="10721836"/>
+        <c:crossAx val="8730332"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2331,7 +2337,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="10721836"/>
+        <c:axId val="8730332"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2373,7 +2379,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="69572257"/>
+        <c:crossAx val="95415480"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2430,12 +2436,12 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>-259920</xdr:colOff>
+      <xdr:colOff>-511560</xdr:colOff>
       <xdr:row>9</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>16</xdr:col>
+      <xdr:col>15</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>1080</xdr:rowOff>
@@ -2446,8 +2452,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-13231080" y="2238480"/>
-        <a:ext cx="5759640" cy="3239640"/>
+        <a:off x="-12871080" y="2238480"/>
+        <a:ext cx="5399640" cy="3239640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2460,15 +2466,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>-262080</xdr:colOff>
+      <xdr:colOff>-785520</xdr:colOff>
       <xdr:row>25</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>7</xdr:col>
+      <xdr:col>8</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>55</xdr:row>
-      <xdr:rowOff>44640</xdr:rowOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>149760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -2476,8 +2482,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="-5900760" y="5477040"/>
-        <a:ext cx="5759640" cy="5759640"/>
+        <a:off x="-7340760" y="5477040"/>
+        <a:ext cx="7199640" cy="3959640"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -22018,7 +22024,7 @@
         <v>225000</v>
       </c>
       <c r="H6" s="28" t="n">
-        <f aca="false">IF(E6=0,0,F6/E6)</f>
+        <f aca="false">IF(OR(B6="",E6=0),"",F6/E6)</f>
         <v>0.25</v>
       </c>
     </row>
@@ -22045,7 +22051,7 @@
         <v>68928</v>
       </c>
       <c r="H7" s="28" t="n">
-        <f aca="false">IF(E7=0,0,F7/E7)</f>
+        <f aca="false">IF(OR(B7="",E7=0),"",F7/E7)</f>
         <v>0.282</v>
       </c>
     </row>
@@ -22072,7 +22078,7 @@
         <v>15214</v>
       </c>
       <c r="H8" s="28" t="n">
-        <f aca="false">IF(E8=0,0,F8/E8)</f>
+        <f aca="false">IF(OR(B8="",E8=0),"",F8/E8)</f>
         <v>0.154777777777778</v>
       </c>
     </row>
@@ -22094,9 +22100,9 @@
         <f aca="false">E9-F9</f>
         <v>0</v>
       </c>
-      <c r="H9" s="28" t="n">
-        <f aca="false">IF(E9=0,0,F9/E9)</f>
-        <v>0</v>
+      <c r="H9" s="28" t="str">
+        <f aca="false">IF(OR(B9="",E9=0),"",F9/E9)</f>
+        <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22117,9 +22123,9 @@
         <f aca="false">E10-F10</f>
         <v>0</v>
       </c>
-      <c r="H10" s="28" t="n">
-        <f aca="false">IF(E10=0,0,F10/E10)</f>
-        <v>0</v>
+      <c r="H10" s="28" t="str">
+        <f aca="false">IF(OR(B10="",E10=0),"",F10/E10)</f>
+        <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22140,9 +22146,9 @@
         <f aca="false">E11-F11</f>
         <v>0</v>
       </c>
-      <c r="H11" s="28" t="n">
-        <f aca="false">IF(E11=0,0,F11/E11)</f>
-        <v>0</v>
+      <c r="H11" s="28" t="str">
+        <f aca="false">IF(OR(B11="",E11=0),"",F11/E11)</f>
+        <v/>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22163,9 +22169,9 @@
         <f aca="false">E12-F12</f>
         <v>0</v>
       </c>
-      <c r="H12" s="28" t="n">
-        <f aca="false">IF(E12=0,0,F12/E12)</f>
-        <v>0</v>
+      <c r="H12" s="28" t="str">
+        <f aca="false">IF(OR(B12="",E12=0),"",F12/E12)</f>
+        <v/>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22186,9 +22192,9 @@
         <f aca="false">E13-F13</f>
         <v>0</v>
       </c>
-      <c r="H13" s="28" t="n">
-        <f aca="false">IF(E13=0,0,F13/E13)</f>
-        <v>0</v>
+      <c r="H13" s="28" t="str">
+        <f aca="false">IF(OR(B13="",E13=0),"",F13/E13)</f>
+        <v/>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22214,7 +22220,7 @@
         <v>63000</v>
       </c>
       <c r="H14" s="28" t="n">
-        <f aca="false">IF(E14=0,0,F14/E14)</f>
+        <f aca="false">IF(OR(B14="",E14=0),"",F14/E14)</f>
         <v>0.25</v>
       </c>
     </row>
@@ -22241,7 +22247,7 @@
         <v>13704</v>
       </c>
       <c r="H15" s="28" t="n">
-        <f aca="false">IF(E15=0,0,F15/E15)</f>
+        <f aca="false">IF(OR(B15="",E15=0),"",F15/E15)</f>
         <v>0.238666666666667</v>
       </c>
     </row>
@@ -22268,7 +22274,7 @@
         <v>53429</v>
       </c>
       <c r="H16" s="28" t="n">
-        <f aca="false">IF(E16=0,0,F16/E16)</f>
+        <f aca="false">IF(OR(B16="",E16=0),"",F16/E16)</f>
         <v>0.257930555555556</v>
       </c>
     </row>
@@ -22295,7 +22301,7 @@
         <v>13642</v>
       </c>
       <c r="H17" s="28" t="n">
-        <f aca="false">IF(E17=0,0,F17/E17)</f>
+        <f aca="false">IF(OR(B17="",E17=0),"",F17/E17)</f>
         <v>0.242111111111111</v>
       </c>
     </row>
@@ -22322,7 +22328,7 @@
         <v>5400</v>
       </c>
       <c r="H18" s="28" t="n">
-        <f aca="false">IF(E18=0,0,F18/E18)</f>
+        <f aca="false">IF(OR(B18="",E18=0),"",F18/E18)</f>
         <v>0.25</v>
       </c>
     </row>
@@ -22349,7 +22355,7 @@
         <v>8480</v>
       </c>
       <c r="H19" s="28" t="n">
-        <f aca="false">IF(E19=0,0,F19/E19)</f>
+        <f aca="false">IF(OR(B19="",E19=0),"",F19/E19)</f>
         <v>0.116666666666667</v>
       </c>
     </row>
@@ -22376,7 +22382,7 @@
         <v>10000</v>
       </c>
       <c r="H20" s="28" t="n">
-        <f aca="false">IF(E20=0,0,F20/E20)</f>
+        <f aca="false">IF(OR(B20="",E20=0),"",F20/E20)</f>
         <v>0.166666666666667</v>
       </c>
     </row>
@@ -22403,7 +22409,7 @@
         <v>10987</v>
       </c>
       <c r="H21" s="28" t="n">
-        <f aca="false">IF(E21=0,0,F21/E21)</f>
+        <f aca="false">IF(OR(B21="",E21=0),"",F21/E21)</f>
         <v>0.237013888888889</v>
       </c>
     </row>
@@ -22430,7 +22436,7 @@
         <v>8400</v>
       </c>
       <c r="H22" s="28" t="n">
-        <f aca="false">IF(E22=0,0,F22/E22)</f>
+        <f aca="false">IF(OR(B22="",E22=0),"",F22/E22)</f>
         <v>0.125</v>
       </c>
     </row>
@@ -22457,7 +22463,7 @@
         <v>3600</v>
       </c>
       <c r="H23" s="28" t="n">
-        <f aca="false">IF(E23=0,0,F23/E23)</f>
+        <f aca="false">IF(OR(B23="",E23=0),"",F23/E23)</f>
         <v>0.25</v>
       </c>
     </row>
@@ -22484,7 +22490,7 @@
         <v>8943</v>
       </c>
       <c r="H24" s="28" t="n">
-        <f aca="false">IF(E24=0,0,F24/E24)</f>
+        <f aca="false">IF(OR(B24="",E24=0),"",F24/E24)</f>
         <v>0.25475</v>
       </c>
     </row>
@@ -22510,9 +22516,9 @@
         <f aca="false">E25-F25</f>
         <v>-5700</v>
       </c>
-      <c r="H25" s="28" t="n">
-        <f aca="false">IF(E25=0,0,F25/E25)</f>
-        <v>0</v>
+      <c r="H25" s="28" t="str">
+        <f aca="false">IF(OR(B25="",E25=0),"",F25/E25)</f>
+        <v/>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22537,9 +22543,9 @@
         <f aca="false">E26-F26</f>
         <v>-5800</v>
       </c>
-      <c r="H26" s="28" t="n">
-        <f aca="false">IF(E26=0,0,F26/E26)</f>
-        <v>0</v>
+      <c r="H26" s="28" t="str">
+        <f aca="false">IF(OR(B26="",E26=0),"",F26/E26)</f>
+        <v/>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22564,9 +22570,9 @@
         <f aca="false">E27-F27</f>
         <v>-2600</v>
       </c>
-      <c r="H27" s="28" t="n">
-        <f aca="false">IF(E27=0,0,F27/E27)</f>
-        <v>0</v>
+      <c r="H27" s="28" t="str">
+        <f aca="false">IF(OR(B27="",E27=0),"",F27/E27)</f>
+        <v/>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22591,9 +22597,9 @@
         <f aca="false">E28-F28</f>
         <v>-2900</v>
       </c>
-      <c r="H28" s="28" t="n">
-        <f aca="false">IF(E28=0,0,F28/E28)</f>
-        <v>0</v>
+      <c r="H28" s="28" t="str">
+        <f aca="false">IF(OR(B28="",E28=0),"",F28/E28)</f>
+        <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22614,9 +22620,9 @@
         <f aca="false">E29-F29</f>
         <v>0</v>
       </c>
-      <c r="H29" s="28" t="n">
-        <f aca="false">IF(E29=0,0,F29/E29)</f>
-        <v>0</v>
+      <c r="H29" s="28" t="str">
+        <f aca="false">IF(OR(B29="",E29=0),"",F29/E29)</f>
+        <v/>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22637,9 +22643,9 @@
         <f aca="false">E30-F30</f>
         <v>0</v>
       </c>
-      <c r="H30" s="28" t="n">
-        <f aca="false">IF(E30=0,0,F30/E30)</f>
-        <v>0</v>
+      <c r="H30" s="28" t="str">
+        <f aca="false">IF(OR(B30="",E30=0),"",F30/E30)</f>
+        <v/>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22660,9 +22666,9 @@
         <f aca="false">E31-F31</f>
         <v>0</v>
       </c>
-      <c r="H31" s="28" t="n">
-        <f aca="false">IF(E31=0,0,F31/E31)</f>
-        <v>0</v>
+      <c r="H31" s="28" t="str">
+        <f aca="false">IF(OR(B31="",E31=0),"",F31/E31)</f>
+        <v/>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22683,9 +22689,9 @@
         <f aca="false">E32-F32</f>
         <v>0</v>
       </c>
-      <c r="H32" s="28" t="n">
-        <f aca="false">IF(E32=0,0,F32/E32)</f>
-        <v>0</v>
+      <c r="H32" s="28" t="str">
+        <f aca="false">IF(OR(B32="",E32=0),"",F32/E32)</f>
+        <v/>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22706,9 +22712,9 @@
         <f aca="false">E33-F33</f>
         <v>0</v>
       </c>
-      <c r="H33" s="28" t="n">
-        <f aca="false">IF(E33=0,0,F33/E33)</f>
-        <v>0</v>
+      <c r="H33" s="28" t="str">
+        <f aca="false">IF(OR(B33="",E33=0),"",F33/E33)</f>
+        <v/>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22729,9 +22735,9 @@
         <f aca="false">E34-F34</f>
         <v>0</v>
       </c>
-      <c r="H34" s="28" t="n">
-        <f aca="false">IF(E34=0,0,F34/E34)</f>
-        <v>0</v>
+      <c r="H34" s="28" t="str">
+        <f aca="false">IF(OR(B34="",E34=0),"",F34/E34)</f>
+        <v/>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22752,9 +22758,9 @@
         <f aca="false">E35-F35</f>
         <v>0</v>
       </c>
-      <c r="H35" s="28" t="n">
-        <f aca="false">IF(E35=0,0,F35/E35)</f>
-        <v>0</v>
+      <c r="H35" s="28" t="str">
+        <f aca="false">IF(OR(B35="",E35=0),"",F35/E35)</f>
+        <v/>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22775,9 +22781,9 @@
         <f aca="false">E36-F36</f>
         <v>0</v>
       </c>
-      <c r="H36" s="28" t="n">
-        <f aca="false">IF(E36=0,0,F36/E36)</f>
-        <v>0</v>
+      <c r="H36" s="28" t="str">
+        <f aca="false">IF(OR(B36="",E36=0),"",F36/E36)</f>
+        <v/>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22798,9 +22804,9 @@
         <f aca="false">E37-F37</f>
         <v>0</v>
       </c>
-      <c r="H37" s="28" t="n">
-        <f aca="false">IF(E37=0,0,F37/E37)</f>
-        <v>0</v>
+      <c r="H37" s="28" t="str">
+        <f aca="false">IF(OR(B37="",E37=0),"",F37/E37)</f>
+        <v/>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22821,9 +22827,9 @@
         <f aca="false">E38-F38</f>
         <v>0</v>
       </c>
-      <c r="H38" s="28" t="n">
-        <f aca="false">IF(E38=0,0,F38/E38)</f>
-        <v>0</v>
+      <c r="H38" s="28" t="str">
+        <f aca="false">IF(OR(B38="",E38=0),"",F38/E38)</f>
+        <v/>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22844,9 +22850,9 @@
         <f aca="false">E39-F39</f>
         <v>0</v>
       </c>
-      <c r="H39" s="28" t="n">
-        <f aca="false">IF(E39=0,0,F39/E39)</f>
-        <v>0</v>
+      <c r="H39" s="28" t="str">
+        <f aca="false">IF(OR(B39="",E39=0),"",F39/E39)</f>
+        <v/>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22867,9 +22873,9 @@
         <f aca="false">E40-F40</f>
         <v>0</v>
       </c>
-      <c r="H40" s="28" t="n">
-        <f aca="false">IF(E40=0,0,F40/E40)</f>
-        <v>0</v>
+      <c r="H40" s="28" t="str">
+        <f aca="false">IF(OR(B40="",E40=0),"",F40/E40)</f>
+        <v/>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22946,7 +22952,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{4734A4A9-B268-4774-9F40-4D3127B14CE7}</x14:id>
+          <x14:id>{99AAF59D-B12B-45D2-91E9-5023DAF054DB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -22963,7 +22969,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{4734A4A9-B268-4774-9F40-4D3127B14CE7}">
+          <x14:cfRule type="dataBar" id="{99AAF59D-B12B-45D2-91E9-5023DAF054DB}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -23374,7 +23380,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{17EF1340-31A8-4D86-87DA-785899FEA038}</x14:id>
+          <x14:id>{203FBE37-6532-4DDE-B353-723FC02AAF16}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -23404,7 +23410,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{17EF1340-31A8-4D86-87DA-785899FEA038}">
+          <x14:cfRule type="dataBar" id="{203FBE37-6532-4DDE-B353-723FC02AAF16}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -23464,7 +23470,7 @@
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
     </row>
-    <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="4" t="s">
         <v>112</v>
       </c>
@@ -23521,14 +23527,22 @@
         <f aca="false">IF(1&gt;cfgRDays,"",cfgRStart+1-1)</f>
         <v>46426</v>
       </c>
-      <c r="J7" s="7"/>
-      <c r="K7" s="6"/>
-      <c r="L7" s="7"/>
-      <c r="M7" s="12"/>
+      <c r="J7" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L7" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M7" s="12" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="32" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C8" s="34" t="n">
         <f aca="true">MAX(0,cfgRStart-TODAY())</f>
@@ -23542,10 +23556,18 @@
         <f aca="false">IF(2&gt;cfgRDays,"",cfgRStart+2-1)</f>
         <v>46427</v>
       </c>
-      <c r="J8" s="7"/>
-      <c r="K8" s="6"/>
-      <c r="L8" s="7"/>
-      <c r="M8" s="12"/>
+      <c r="J8" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L8" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M8" s="12" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="H9" s="26" t="n">
@@ -23556,14 +23578,22 @@
         <f aca="false">IF(3&gt;cfgRDays,"",cfgRStart+3-1)</f>
         <v>46428</v>
       </c>
-      <c r="J9" s="7"/>
-      <c r="K9" s="6"/>
-      <c r="L9" s="7"/>
-      <c r="M9" s="12"/>
-    </row>
-    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="J9" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K9" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L9" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M9" s="12" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="35" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C10" s="35"/>
       <c r="D10" s="35"/>
@@ -23577,20 +23607,28 @@
         <f aca="false">IF(4&gt;cfgRDays,"",cfgRStart+4-1)</f>
         <v>46429</v>
       </c>
-      <c r="J10" s="7"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="7"/>
-      <c r="M10" s="12"/>
-    </row>
-    <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="J10" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K10" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L10" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M10" s="12" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="4" t="s">
         <v>49</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>94</v>
@@ -23606,10 +23644,18 @@
         <f aca="false">IF(5&gt;cfgRDays,"",cfgRStart+5-1)</f>
         <v>46430</v>
       </c>
-      <c r="J11" s="7"/>
-      <c r="K11" s="6"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="12"/>
+      <c r="J11" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K11" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L11" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="M11" s="12" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="24" t="s">
@@ -23627,7 +23673,7 @@
         <v>-700</v>
       </c>
       <c r="F12" s="28" t="n">
-        <f aca="false">IF(N(C12)=0,0,D12/C12)</f>
+        <f aca="false">IF(N(C12)=0,"",D12/C12)</f>
         <v>1.14</v>
       </c>
       <c r="H12" s="26" t="n">
@@ -23638,10 +23684,18 @@
         <f aca="false">IF(6&gt;cfgRDays,"",cfgRStart+6-1)</f>
         <v>46431</v>
       </c>
-      <c r="J12" s="7"/>
-      <c r="K12" s="6"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="12"/>
+      <c r="J12" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K12" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L12" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M12" s="12" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="24" t="s">
@@ -23659,7 +23713,7 @@
         <v>200</v>
       </c>
       <c r="F13" s="28" t="n">
-        <f aca="false">IF(N(C13)=0,0,D13/C13)</f>
+        <f aca="false">IF(N(C13)=0,"",D13/C13)</f>
         <v>0.966666666666667</v>
       </c>
       <c r="H13" s="26" t="n">
@@ -23670,10 +23724,18 @@
         <f aca="false">IF(7&gt;cfgRDays,"",cfgRStart+7-1)</f>
         <v>46432</v>
       </c>
-      <c r="J13" s="7"/>
-      <c r="K13" s="6"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="12"/>
+      <c r="J13" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L13" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M13" s="12" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="24" t="s">
@@ -23691,7 +23753,7 @@
         <v>400</v>
       </c>
       <c r="F14" s="28" t="n">
-        <f aca="false">IF(N(C14)=0,0,D14/C14)</f>
+        <f aca="false">IF(N(C14)=0,"",D14/C14)</f>
         <v>0.866666666666667</v>
       </c>
       <c r="H14" s="26" t="n">
@@ -23702,10 +23764,18 @@
         <f aca="false">IF(8&gt;cfgRDays,"",cfgRStart+8-1)</f>
         <v>46433</v>
       </c>
-      <c r="J14" s="7"/>
-      <c r="K14" s="6"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="12"/>
+      <c r="J14" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L14" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M14" s="12" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="24" t="s">
@@ -23723,7 +23793,7 @@
         <v>-400</v>
       </c>
       <c r="F15" s="28" t="n">
-        <f aca="false">IF(N(C15)=0,0,D15/C15)</f>
+        <f aca="false">IF(N(C15)=0,"",D15/C15)</f>
         <v>1.16</v>
       </c>
       <c r="H15" s="26" t="n">
@@ -23734,10 +23804,18 @@
         <f aca="false">IF(9&gt;cfgRDays,"",cfgRStart+9-1)</f>
         <v>46434</v>
       </c>
-      <c r="J15" s="7"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="12"/>
+      <c r="J15" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L15" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="M15" s="12" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="24"/>
@@ -23750,9 +23828,9 @@
         <f aca="false">N(C16)-D16</f>
         <v>0</v>
       </c>
-      <c r="F16" s="28" t="n">
-        <f aca="false">IF(N(C16)=0,0,D16/C16)</f>
-        <v>0</v>
+      <c r="F16" s="28" t="str">
+        <f aca="false">IF(N(C16)=0,"",D16/C16)</f>
+        <v/>
       </c>
       <c r="H16" s="26" t="n">
         <f aca="false">IF(10&gt;cfgRDays,"",10)</f>
@@ -23762,10 +23840,18 @@
         <f aca="false">IF(10&gt;cfgRDays,"",cfgRStart+10-1)</f>
         <v>46435</v>
       </c>
-      <c r="J16" s="7"/>
-      <c r="K16" s="6"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="12"/>
+      <c r="J16" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L16" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M16" s="12" t="n">
+        <v>150</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="24"/>
@@ -23778,9 +23864,9 @@
         <f aca="false">N(C17)-D17</f>
         <v>0</v>
       </c>
-      <c r="F17" s="28" t="n">
-        <f aca="false">IF(N(C17)=0,0,D17/C17)</f>
-        <v>0</v>
+      <c r="F17" s="28" t="str">
+        <f aca="false">IF(N(C17)=0,"",D17/C17)</f>
+        <v/>
       </c>
       <c r="H17" s="26" t="n">
         <f aca="false">IF(11&gt;cfgRDays,"",11)</f>
@@ -23790,10 +23876,18 @@
         <f aca="false">IF(11&gt;cfgRDays,"",cfgRStart+11-1)</f>
         <v>46436</v>
       </c>
-      <c r="J17" s="7"/>
-      <c r="K17" s="6"/>
-      <c r="L17" s="7"/>
-      <c r="M17" s="12"/>
+      <c r="J17" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="L17" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M17" s="12" t="n">
+        <v>200</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="24"/>
@@ -23806,9 +23900,9 @@
         <f aca="false">N(C18)-D18</f>
         <v>0</v>
       </c>
-      <c r="F18" s="28" t="n">
-        <f aca="false">IF(N(C18)=0,0,D18/C18)</f>
-        <v>0</v>
+      <c r="F18" s="28" t="str">
+        <f aca="false">IF(N(C18)=0,"",D18/C18)</f>
+        <v/>
       </c>
       <c r="H18" s="26" t="n">
         <f aca="false">IF(12&gt;cfgRDays,"",12)</f>
@@ -23818,10 +23912,18 @@
         <f aca="false">IF(12&gt;cfgRDays,"",cfgRStart+12-1)</f>
         <v>46437</v>
       </c>
-      <c r="J18" s="7"/>
-      <c r="K18" s="6"/>
-      <c r="L18" s="7"/>
-      <c r="M18" s="12"/>
+      <c r="J18" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L18" s="7" t="s">
+        <v>119</v>
+      </c>
+      <c r="M18" s="12" t="n">
+        <v>50</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="24"/>
@@ -23834,9 +23936,9 @@
         <f aca="false">N(C19)-D19</f>
         <v>0</v>
       </c>
-      <c r="F19" s="28" t="n">
-        <f aca="false">IF(N(C19)=0,0,D19/C19)</f>
-        <v>0</v>
+      <c r="F19" s="28" t="str">
+        <f aca="false">IF(N(C19)=0,"",D19/C19)</f>
+        <v/>
       </c>
       <c r="H19" s="26" t="n">
         <f aca="false">IF(13&gt;cfgRDays,"",13)</f>
@@ -23886,7 +23988,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="32" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="D21" s="36" t="n">
         <f aca="false">SUMIFS(txAmt,txType,"مصروف",txDate,"&gt;="&amp;cfgRStart,txDate,"&lt;="&amp;cfgREnd)</f>
@@ -23919,9 +24021,9 @@
       <c r="L22" s="7"/>
       <c r="M22" s="12"/>
     </row>
-    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="37" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C23" s="37"/>
       <c r="H23" s="26" t="n">
@@ -23939,7 +24041,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="38" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C24" s="12" t="n">
         <v>350000</v>
@@ -23959,7 +24061,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="38" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C25" s="12" t="n">
         <v>120000</v>
@@ -23979,7 +24081,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="38" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="C26" s="12" t="n">
         <v>80000</v>
@@ -23999,7 +24101,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="38" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C27" s="12" t="n">
         <v>20000</v>
@@ -24019,7 +24121,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="38" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="C28" s="12" t="n">
         <v>30000</v>
@@ -24039,7 +24141,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="32" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="C29" s="36" t="n">
         <f aca="false">C24+C25+C26+C27-C28</f>
@@ -24060,7 +24162,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="32" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C30" s="36" t="n">
         <f aca="false">cfgNisab</f>
@@ -24081,7 +24183,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="32" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C31" s="39" t="str">
         <f aca="false">IF(C29&gt;=C30,"نعم","لا")</f>
@@ -24102,7 +24204,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="32" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="C32" s="22" t="n">
         <f aca="false">IF(C29&gt;=C30,C29*0.025,0)</f>
@@ -24137,7 +24239,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B34" s="40" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C34" s="40"/>
       <c r="D34" s="40"/>
@@ -24196,19 +24298,19 @@
       <c r="I37" s="41"/>
       <c r="J37" s="21" t="str">
         <f aca="false">COUNTIF(J7:J36,"✓")&amp;" / "&amp;cfgRDays</f>
-        <v>0 / 30</v>
+        <v>12 / 30</v>
       </c>
       <c r="K37" s="42" t="n">
         <f aca="false">SUM(K7:K36)</f>
-        <v>0</v>
+        <v>220</v>
       </c>
       <c r="L37" s="21" t="str">
         <f aca="false">COUNTIF(L7:L36,"✓")&amp;" / "&amp;cfgRDays</f>
-        <v>0 / 30</v>
+        <v>10 / 30</v>
       </c>
       <c r="M37" s="22" t="n">
         <f aca="false">SUM(M7:M36)</f>
-        <v>0</v>
+        <v>1500</v>
       </c>
     </row>
   </sheetData>
@@ -24226,7 +24328,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{365B5428-3BF9-45F7-AFD2-F5F84E47A8C3}</x14:id>
+          <x14:id>{456DC181-6A6A-4AA2-B9C6-FB12B486EFB3}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -24252,7 +24354,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{365B5428-3BF9-45F7-AFD2-F5F84E47A8C3}">
+          <x14:cfRule type="dataBar" id="{456DC181-6A6A-4AA2-B9C6-FB12B486EFB3}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>